<commit_message>
Case documents for John Doe v. Robert Smith: spec, renderer, audit, wiring (in progress)
The Case Flow's own document set (documents/case-flow/, RS01–RS60), in
progress: the spec of every document's facts, plants and trainer key
(build/case-flow/documents/SPEC.md), the HTML → PDF renderer, the audit
that reads every PDF back against case-file.md, the metadata and each
activity's documents (js/cm-case-flow-docs.js), the Documents page and
the "Work from" line on each activity, the CI data check, and the Net
Sheet's Robert Smith practice tab (the Apex tab kept, archived). The
document sources are being written; the set is completed in the next
commit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01So6RsHEAxqg1h82DoqaUJQ
</commit_message>
<xml_diff>
--- a/documents/templates/LSH_Net_Sheet_v2_FIXED.xlsx
+++ b/documents/templates/LSH_Net_Sheet_v2_FIXED.xlsx
@@ -4,7 +4,8 @@
   <workbookPr/>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LSH Net Sheet" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="John Doe Practice" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Robert Smith Practice" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Apex Practice (archived)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1582,6 +1583,1150 @@
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve"> PRACTICE — John Doe v. Robert Smith (Track A: all three layers paid at limits). Fill the yellow cells; verify every figure against the source documents (RS22–RS26, RS31, RS41, RS42, RS44).</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+    </row>
+    <row r="2">
+      <c r="B2" s="3" t="n"/>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>1. SETTLEMENT RECOVERY SUMMARY</t>
+        </is>
+      </c>
+      <c r="C5" s="25" t="n"/>
+      <c r="D5" s="25" t="n"/>
+      <c r="E5" s="25" t="n"/>
+      <c r="F5" s="25" t="n"/>
+      <c r="G5" s="25" t="n"/>
+      <c r="H5" s="25" t="n"/>
+      <c r="I5" s="25" t="n"/>
+      <c r="J5" s="25" t="n"/>
+      <c r="K5" s="25" t="n"/>
+      <c r="L5" s="26" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="n"/>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="25" t="n"/>
+      <c r="F6" s="25" t="n"/>
+      <c r="G6" s="25" t="n"/>
+      <c r="H6" s="25" t="n"/>
+      <c r="I6" s="25" t="n"/>
+      <c r="J6" s="25" t="n"/>
+      <c r="K6" s="26" t="n"/>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="7" t="n"/>
+      <c r="O6" s="7" t="n"/>
+      <c r="P6" s="7" t="n"/>
+      <c r="Q6" s="7" t="n"/>
+      <c r="R6" s="7" t="n"/>
+      <c r="S6" s="7" t="n"/>
+      <c r="T6" s="7" t="n"/>
+      <c r="U6" s="7" t="n"/>
+      <c r="V6" s="7" t="n"/>
+      <c r="W6" s="7" t="n"/>
+      <c r="X6" s="7" t="n"/>
+      <c r="Y6" s="7" t="n"/>
+      <c r="Z6" s="7" t="n"/>
+      <c r="AA6" s="7" t="n"/>
+      <c r="AB6" s="7" t="n"/>
+      <c r="AC6" s="7" t="n"/>
+      <c r="AD6" s="7" t="n"/>
+      <c r="AE6" s="7" t="n"/>
+      <c r="AF6" s="7" t="n"/>
+      <c r="AG6" s="7" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>Gross Settlement</t>
+        </is>
+      </c>
+      <c r="C7" s="22" t="inlineStr">
+        <is>
+          <t>Keystone BI $10,000 (KM-26-440871) + Harbor Point UM $20,000 (HP-26-7741) + Cardinal State UM $10,000 (CS-26-20355)</t>
+        </is>
+      </c>
+      <c r="D7" s="25" t="n"/>
+      <c r="E7" s="25" t="n"/>
+      <c r="F7" s="25" t="n"/>
+      <c r="G7" s="25" t="n"/>
+      <c r="H7" s="25" t="n"/>
+      <c r="I7" s="25" t="n"/>
+      <c r="J7" s="25" t="n"/>
+      <c r="K7" s="26" t="n"/>
+      <c r="L7" s="14" t="n">
+        <v>40000</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="24" t="inlineStr">
+        <is>
+          <t>2. ATTORNEY FEES &amp; ADVANCED CASE EXPENSES</t>
+        </is>
+      </c>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="25" t="n"/>
+      <c r="F9" s="25" t="n"/>
+      <c r="G9" s="25" t="n"/>
+      <c r="H9" s="25" t="n"/>
+      <c r="I9" s="25" t="n"/>
+      <c r="J9" s="25" t="n"/>
+      <c r="K9" s="25" t="n"/>
+      <c r="L9" s="26" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="n"/>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Expense Type</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="25" t="n"/>
+      <c r="G10" s="25" t="n"/>
+      <c r="H10" s="25" t="n"/>
+      <c r="I10" s="25" t="n"/>
+      <c r="J10" s="25" t="n"/>
+      <c r="K10" s="26" t="n"/>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="7" t="n"/>
+      <c r="O10" s="7" t="n"/>
+      <c r="P10" s="7" t="n"/>
+      <c r="Q10" s="7" t="n"/>
+      <c r="R10" s="7" t="n"/>
+      <c r="S10" s="7" t="n"/>
+      <c r="T10" s="7" t="n"/>
+      <c r="U10" s="7" t="n"/>
+      <c r="V10" s="7" t="n"/>
+      <c r="W10" s="7" t="n"/>
+      <c r="X10" s="7" t="n"/>
+      <c r="Y10" s="7" t="n"/>
+      <c r="Z10" s="7" t="n"/>
+      <c r="AA10" s="7" t="n"/>
+      <c r="AB10" s="7" t="n"/>
+      <c r="AC10" s="7" t="n"/>
+      <c r="AD10" s="7" t="n"/>
+      <c r="AE10" s="7" t="n"/>
+      <c r="AF10" s="7" t="n"/>
+      <c r="AG10" s="7" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="22" t="inlineStr">
+        <is>
+          <t>Attorney Fees</t>
+        </is>
+      </c>
+      <c r="C11" s="27" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="D11" s="25" t="n"/>
+      <c r="E11" s="25" t="n"/>
+      <c r="F11" s="25" t="n"/>
+      <c r="G11" s="25" t="n"/>
+      <c r="H11" s="25" t="n"/>
+      <c r="I11" s="25" t="n"/>
+      <c r="J11" s="25" t="n"/>
+      <c r="K11" s="26" t="n"/>
+      <c r="L11" s="14">
+        <f>L7*C11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>Filing fees &amp; Summons</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
+      <c r="F12" s="25" t="n"/>
+      <c r="G12" s="25" t="n"/>
+      <c r="H12" s="25" t="n"/>
+      <c r="I12" s="25" t="n"/>
+      <c r="J12" s="25" t="n"/>
+      <c r="K12" s="26" t="n"/>
+      <c r="L12" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>Process Server</t>
+        </is>
+      </c>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
+      <c r="F13" s="25" t="n"/>
+      <c r="G13" s="25" t="n"/>
+      <c r="H13" s="25" t="n"/>
+      <c r="I13" s="25" t="n"/>
+      <c r="J13" s="25" t="n"/>
+      <c r="K13" s="26" t="n"/>
+      <c r="L13" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="22" t="inlineStr">
+        <is>
+          <t>Mediation</t>
+        </is>
+      </c>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="25" t="n"/>
+      <c r="E14" s="25" t="n"/>
+      <c r="F14" s="25" t="n"/>
+      <c r="G14" s="25" t="n"/>
+      <c r="H14" s="25" t="n"/>
+      <c r="I14" s="25" t="n"/>
+      <c r="J14" s="25" t="n"/>
+      <c r="K14" s="26" t="n"/>
+      <c r="L14" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="22" t="inlineStr">
+        <is>
+          <t>CME Videographer</t>
+        </is>
+      </c>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
+      <c r="F15" s="25" t="n"/>
+      <c r="G15" s="25" t="n"/>
+      <c r="H15" s="25" t="n"/>
+      <c r="I15" s="25" t="n"/>
+      <c r="J15" s="25" t="n"/>
+      <c r="K15" s="26" t="n"/>
+      <c r="L15" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="22" t="inlineStr">
+        <is>
+          <t>Deposition</t>
+        </is>
+      </c>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="25" t="n"/>
+      <c r="E16" s="25" t="n"/>
+      <c r="F16" s="25" t="n"/>
+      <c r="G16" s="25" t="n"/>
+      <c r="H16" s="25" t="n"/>
+      <c r="I16" s="25" t="n"/>
+      <c r="J16" s="25" t="n"/>
+      <c r="K16" s="26" t="n"/>
+      <c r="L16" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>Postage</t>
+        </is>
+      </c>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
+      <c r="F17" s="25" t="n"/>
+      <c r="G17" s="25" t="n"/>
+      <c r="H17" s="25" t="n"/>
+      <c r="I17" s="25" t="n"/>
+      <c r="J17" s="25" t="n"/>
+      <c r="K17" s="26" t="n"/>
+      <c r="L17" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>Medical records/bills req.</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
+      <c r="F18" s="25" t="n"/>
+      <c r="G18" s="25" t="n"/>
+      <c r="H18" s="25" t="n"/>
+      <c r="I18" s="25" t="n"/>
+      <c r="J18" s="25" t="n"/>
+      <c r="K18" s="26" t="n"/>
+      <c r="L18" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="22" t="inlineStr">
+        <is>
+          <t>File Storage fee</t>
+        </is>
+      </c>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
+      <c r="F19" s="25" t="n"/>
+      <c r="G19" s="25" t="n"/>
+      <c r="H19" s="25" t="n"/>
+      <c r="I19" s="25" t="n"/>
+      <c r="J19" s="25" t="n"/>
+      <c r="K19" s="26" t="n"/>
+      <c r="L19" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="28" t="inlineStr">
+        <is>
+          <t>Total Attorney Costs</t>
+        </is>
+      </c>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
+      <c r="F20" s="25" t="n"/>
+      <c r="G20" s="25" t="n"/>
+      <c r="H20" s="25" t="n"/>
+      <c r="I20" s="25" t="n"/>
+      <c r="J20" s="25" t="n"/>
+      <c r="K20" s="26" t="n"/>
+      <c r="L20" s="17">
+        <f>SUM(L12:L19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="28" t="inlineStr">
+        <is>
+          <t>Total Fees &amp; Costs</t>
+        </is>
+      </c>
+      <c r="C21" s="25" t="n"/>
+      <c r="D21" s="25" t="n"/>
+      <c r="E21" s="25" t="n"/>
+      <c r="F21" s="25" t="n"/>
+      <c r="G21" s="25" t="n"/>
+      <c r="H21" s="25" t="n"/>
+      <c r="I21" s="25" t="n"/>
+      <c r="J21" s="25" t="n"/>
+      <c r="K21" s="26" t="n"/>
+      <c r="L21" s="17">
+        <f>L11+L20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>3. MEDICAL PROVIDER LEDGER &amp; LIEN REDUCTIONS</t>
+        </is>
+      </c>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
+      <c r="F23" s="25" t="n"/>
+      <c r="G23" s="25" t="n"/>
+      <c r="H23" s="25" t="n"/>
+      <c r="I23" s="25" t="n"/>
+      <c r="J23" s="25" t="n"/>
+      <c r="K23" s="25" t="n"/>
+      <c r="L23" s="26" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="n"/>
+      <c r="B24" s="8" t="inlineStr">
+        <is>
+          <t>Provider Type</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Provider Name</t>
+        </is>
+      </c>
+      <c r="D24" s="18" t="inlineStr">
+        <is>
+          <t>Total Charges</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>PIP Payments</t>
+        </is>
+      </c>
+      <c r="F24" s="8" t="inlineStr">
+        <is>
+          <t>Health Payments</t>
+        </is>
+      </c>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Med Pay</t>
+        </is>
+      </c>
+      <c r="H24" s="8" t="inlineStr">
+        <is>
+          <t>Adjustments</t>
+        </is>
+      </c>
+      <c r="I24" s="8" t="inlineStr">
+        <is>
+          <t>Balance Owed</t>
+        </is>
+      </c>
+      <c r="J24" s="19" t="inlineStr">
+        <is>
+          <t>Max Offer</t>
+        </is>
+      </c>
+      <c r="K24" s="19" t="inlineStr">
+        <is>
+          <t>Low Offer</t>
+        </is>
+      </c>
+      <c r="L24" s="8" t="inlineStr">
+        <is>
+          <t>Reduced Bill</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="7" t="n"/>
+      <c r="O24" s="7" t="n"/>
+      <c r="P24" s="7" t="n"/>
+      <c r="Q24" s="7" t="n"/>
+      <c r="R24" s="7" t="n"/>
+      <c r="S24" s="7" t="n"/>
+      <c r="T24" s="7" t="n"/>
+      <c r="U24" s="7" t="n"/>
+      <c r="V24" s="7" t="n"/>
+      <c r="W24" s="7" t="n"/>
+      <c r="X24" s="7" t="n"/>
+      <c r="Y24" s="7" t="n"/>
+      <c r="Z24" s="7" t="n"/>
+      <c r="AA24" s="7" t="n"/>
+      <c r="AB24" s="7" t="n"/>
+      <c r="AC24" s="7" t="n"/>
+      <c r="AD24" s="7" t="n"/>
+      <c r="AE24" s="7" t="n"/>
+      <c r="AF24" s="7" t="n"/>
+      <c r="AG24" s="7" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>Urgent care</t>
+        </is>
+      </c>
+      <c r="C25" s="22" t="inlineStr">
+        <is>
+          <t>Riverton Urgent Care (DOS 02/20/2026)</t>
+        </is>
+      </c>
+      <c r="D25" s="14" t="n">
+        <v>685</v>
+      </c>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="30" t="n"/>
+      <c r="G25" s="30" t="n">
+        <v>685</v>
+      </c>
+      <c r="H25" s="30" t="n"/>
+      <c r="I25" s="14">
+        <f>D25-E25-F25-G25-H25</f>
+        <v/>
+      </c>
+      <c r="J25" s="30" t="n"/>
+      <c r="K25" s="30" t="n"/>
+      <c r="L25" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>Chiro / PT (LOP)</t>
+        </is>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Riverton Spine &amp; Rehab — itemized LOP ledger as billed</t>
+        </is>
+      </c>
+      <c r="D26" s="14" t="n">
+        <v>6290</v>
+      </c>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="30" t="n"/>
+      <c r="G26" s="30" t="n"/>
+      <c r="H26" s="30" t="n"/>
+      <c r="I26" s="14">
+        <f>D26-E26-F26-G26-H26</f>
+        <v/>
+      </c>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="30" t="n"/>
+      <c r="L26" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="22" t="inlineStr">
+        <is>
+          <t>Orthopedics</t>
+        </is>
+      </c>
+      <c r="C27" s="22" t="inlineStr">
+        <is>
+          <t>Lakeside Orthopedics (3 visits)</t>
+        </is>
+      </c>
+      <c r="D27" s="14" t="n">
+        <v>1920</v>
+      </c>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="30" t="n"/>
+      <c r="G27" s="30" t="n">
+        <v>1920</v>
+      </c>
+      <c r="H27" s="30" t="n"/>
+      <c r="I27" s="14">
+        <f>D27-E27-F27-G27-H27</f>
+        <v/>
+      </c>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="30" t="n"/>
+      <c r="L27" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="22" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="C28" s="22" t="inlineStr">
+        <is>
+          <t>Summit Imaging Center (cervical MRI 03/13/2026)</t>
+        </is>
+      </c>
+      <c r="D28" s="14" t="n">
+        <v>2395</v>
+      </c>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="30" t="n"/>
+      <c r="G28" s="30" t="n">
+        <v>2395</v>
+      </c>
+      <c r="H28" s="30" t="n"/>
+      <c r="I28" s="14">
+        <f>D28-E28-F28-G28-H28</f>
+        <v/>
+      </c>
+      <c r="J28" s="30" t="n"/>
+      <c r="K28" s="30" t="n"/>
+      <c r="L28" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="22" t="inlineStr">
+        <is>
+          <t>Pain management</t>
+        </is>
+      </c>
+      <c r="C29" s="22" t="inlineStr">
+        <is>
+          <t>Crescent Pain &amp; Spine (ESI 05/15/2026)</t>
+        </is>
+      </c>
+      <c r="D29" s="14" t="n">
+        <v>3400</v>
+      </c>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="30" t="n">
+        <v>1860</v>
+      </c>
+      <c r="G29" s="30" t="n"/>
+      <c r="H29" s="30" t="n">
+        <v>1540</v>
+      </c>
+      <c r="I29" s="14">
+        <f>D29-E29-F29-G29-H29</f>
+        <v/>
+      </c>
+      <c r="J29" s="30" t="n"/>
+      <c r="K29" s="30" t="n"/>
+      <c r="L29" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="22" t="inlineStr">
+        <is>
+          <t>Health plan lien (verify!)</t>
+        </is>
+      </c>
+      <c r="C30" s="22" t="inlineStr">
+        <is>
+          <t>Peach State Health Plan reimbursement claim — fully insured group plan</t>
+        </is>
+      </c>
+      <c r="D30" s="14" t="n">
+        <v>1860</v>
+      </c>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="30" t="n"/>
+      <c r="G30" s="30" t="n"/>
+      <c r="H30" s="30" t="n"/>
+      <c r="I30" s="14">
+        <f>D30-E30-F30-G30-H30</f>
+        <v/>
+      </c>
+      <c r="J30" s="30" t="n"/>
+      <c r="K30" s="30" t="n"/>
+      <c r="L30" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
+      <c r="G31" s="14" t="n"/>
+      <c r="H31" s="14" t="n"/>
+      <c r="I31" s="14">
+        <f>D31-E31-F31-G31-H31</f>
+        <v/>
+      </c>
+      <c r="J31" s="14" t="n"/>
+      <c r="K31" s="14" t="n"/>
+      <c r="L31" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="14" t="n"/>
+      <c r="E32" s="14" t="n"/>
+      <c r="F32" s="14" t="n"/>
+      <c r="G32" s="14" t="n"/>
+      <c r="H32" s="14" t="n"/>
+      <c r="I32" s="14">
+        <f>D32-E32-F32-G32-H32</f>
+        <v/>
+      </c>
+      <c r="J32" s="14" t="n"/>
+      <c r="K32" s="14" t="n"/>
+      <c r="L32" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="14" t="n"/>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="14" t="n"/>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="14" t="n"/>
+      <c r="I33" s="14">
+        <f>D33-E33-F33-G33-H33</f>
+        <v/>
+      </c>
+      <c r="J33" s="14" t="n"/>
+      <c r="K33" s="14" t="n"/>
+      <c r="L33" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="14" t="n"/>
+      <c r="E34" s="14" t="n"/>
+      <c r="F34" s="14" t="n"/>
+      <c r="G34" s="14" t="n"/>
+      <c r="H34" s="14" t="n"/>
+      <c r="I34" s="14">
+        <f>D34-E34-F34-G34-H34</f>
+        <v/>
+      </c>
+      <c r="J34" s="14" t="n"/>
+      <c r="K34" s="14" t="n"/>
+      <c r="L34" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="14" t="n"/>
+      <c r="E35" s="14" t="n"/>
+      <c r="F35" s="14" t="n"/>
+      <c r="G35" s="14" t="n"/>
+      <c r="H35" s="14" t="n"/>
+      <c r="I35" s="14">
+        <f>D35-E35-F35-G35-H35</f>
+        <v/>
+      </c>
+      <c r="J35" s="14" t="n"/>
+      <c r="K35" s="14" t="n"/>
+      <c r="L35" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="14" t="n"/>
+      <c r="E36" s="14" t="n"/>
+      <c r="F36" s="14" t="n"/>
+      <c r="G36" s="14" t="n"/>
+      <c r="H36" s="14" t="n"/>
+      <c r="I36" s="14">
+        <f>D36-E36-F36-G36-H36</f>
+        <v/>
+      </c>
+      <c r="J36" s="14" t="n"/>
+      <c r="K36" s="14" t="n"/>
+      <c r="L36" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="14" t="n"/>
+      <c r="E37" s="14" t="n"/>
+      <c r="F37" s="14" t="n"/>
+      <c r="G37" s="14" t="n"/>
+      <c r="H37" s="14" t="n"/>
+      <c r="I37" s="14">
+        <f>D37-E37-F37-G37-H37</f>
+        <v/>
+      </c>
+      <c r="J37" s="14" t="n"/>
+      <c r="K37" s="14" t="n"/>
+      <c r="L37" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="14" t="n"/>
+      <c r="E38" s="14" t="n"/>
+      <c r="F38" s="14" t="n"/>
+      <c r="G38" s="14" t="n"/>
+      <c r="H38" s="14" t="n"/>
+      <c r="I38" s="14">
+        <f>D38-E38-F38-G38-H38</f>
+        <v/>
+      </c>
+      <c r="J38" s="14" t="n"/>
+      <c r="K38" s="14" t="n"/>
+      <c r="L38" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="14" t="n"/>
+      <c r="E39" s="14" t="n"/>
+      <c r="F39" s="14" t="n"/>
+      <c r="G39" s="14" t="n"/>
+      <c r="H39" s="14" t="n"/>
+      <c r="I39" s="14">
+        <f>D39-E39-F39-G39-H39</f>
+        <v/>
+      </c>
+      <c r="J39" s="14" t="n"/>
+      <c r="K39" s="14" t="n"/>
+      <c r="L39" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="B40" s="22" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="14" t="n"/>
+      <c r="E40" s="14" t="n"/>
+      <c r="F40" s="14" t="n"/>
+      <c r="G40" s="14" t="n"/>
+      <c r="H40" s="14" t="n"/>
+      <c r="I40" s="14">
+        <f>D40-E40-F40-G40-H40</f>
+        <v/>
+      </c>
+      <c r="J40" s="14" t="n"/>
+      <c r="K40" s="14" t="n"/>
+      <c r="L40" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="B41" s="29" t="n"/>
+      <c r="C41" s="25" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
+      <c r="F41" s="25" t="n"/>
+      <c r="G41" s="26" t="n"/>
+      <c r="H41" s="21" t="n"/>
+      <c r="I41" s="21" t="n"/>
+      <c r="J41" s="21" t="n"/>
+      <c r="K41" s="21" t="n"/>
+      <c r="L41" s="21" t="n"/>
+    </row>
+    <row r="42">
+      <c r="B42" s="22" t="inlineStr">
+        <is>
+          <t>Pre-Settlement Funding</t>
+        </is>
+      </c>
+      <c r="C42" s="22" t="inlineStr">
+        <is>
+          <t>None reported</t>
+        </is>
+      </c>
+      <c r="D42" s="14" t="n"/>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="14" t="n"/>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="14" t="n"/>
+      <c r="I42" s="14">
+        <f>D42-E42-F42-G42-H42</f>
+        <v/>
+      </c>
+      <c r="J42" s="14" t="n"/>
+      <c r="K42" s="14" t="n"/>
+      <c r="L42" s="14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" s="22" t="inlineStr">
+        <is>
+          <t>Prior Attorney</t>
+        </is>
+      </c>
+      <c r="C43" s="22" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="D43" s="14" t="n"/>
+      <c r="E43" s="14" t="n"/>
+      <c r="F43" s="30" t="n"/>
+      <c r="G43" s="30" t="n"/>
+      <c r="H43" s="30" t="n"/>
+      <c r="I43" s="14">
+        <f>D43-E43-F43-G43-H43</f>
+        <v/>
+      </c>
+      <c r="J43" s="30" t="n"/>
+      <c r="K43" s="30" t="n"/>
+      <c r="L43" s="30" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="28" t="inlineStr">
+        <is>
+          <t>Total Liens &amp; Reductions</t>
+        </is>
+      </c>
+      <c r="C44" s="25" t="n"/>
+      <c r="D44" s="25" t="n"/>
+      <c r="E44" s="25" t="n"/>
+      <c r="F44" s="25" t="n"/>
+      <c r="G44" s="25" t="n"/>
+      <c r="H44" s="26" t="n"/>
+      <c r="I44" s="17">
+        <f>SUM(I25:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="17">
+        <f>SUM(J25:J43)</f>
+        <v/>
+      </c>
+      <c r="K44" s="17">
+        <f>SUM(K25:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="17">
+        <f>SUM(L25:L43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" s="24" t="inlineStr">
+        <is>
+          <t>4. FINAL CLIENT DISBURSEMENT CALCULATION</t>
+        </is>
+      </c>
+      <c r="C46" s="25" t="n"/>
+      <c r="D46" s="25" t="n"/>
+      <c r="E46" s="25" t="n"/>
+      <c r="F46" s="25" t="n"/>
+      <c r="G46" s="25" t="n"/>
+      <c r="H46" s="25" t="n"/>
+      <c r="I46" s="25" t="n"/>
+      <c r="J46" s="25" t="n"/>
+      <c r="K46" s="25" t="n"/>
+      <c r="L46" s="26" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="7" t="n"/>
+      <c r="B47" s="8" t="inlineStr">
+        <is>
+          <t>Calculation</t>
+        </is>
+      </c>
+      <c r="C47" s="25" t="n"/>
+      <c r="D47" s="25" t="n"/>
+      <c r="E47" s="25" t="n"/>
+      <c r="F47" s="25" t="n"/>
+      <c r="G47" s="25" t="n"/>
+      <c r="H47" s="25" t="n"/>
+      <c r="I47" s="25" t="n"/>
+      <c r="J47" s="25" t="n"/>
+      <c r="K47" s="26" t="n"/>
+      <c r="L47" s="8" t="inlineStr">
+        <is>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="7" t="n"/>
+      <c r="O47" s="7" t="n"/>
+      <c r="P47" s="7" t="n"/>
+      <c r="Q47" s="7" t="n"/>
+      <c r="R47" s="7" t="n"/>
+      <c r="S47" s="7" t="n"/>
+      <c r="T47" s="7" t="n"/>
+      <c r="U47" s="7" t="n"/>
+      <c r="V47" s="7" t="n"/>
+      <c r="W47" s="7" t="n"/>
+      <c r="X47" s="7" t="n"/>
+      <c r="Y47" s="7" t="n"/>
+      <c r="Z47" s="7" t="n"/>
+      <c r="AA47" s="7" t="n"/>
+      <c r="AB47" s="7" t="n"/>
+      <c r="AC47" s="7" t="n"/>
+      <c r="AD47" s="7" t="n"/>
+      <c r="AE47" s="7" t="n"/>
+      <c r="AF47" s="7" t="n"/>
+      <c r="AG47" s="7" t="n"/>
+    </row>
+    <row r="48">
+      <c r="B48" s="22" t="inlineStr">
+        <is>
+          <t>Gross Settlement</t>
+        </is>
+      </c>
+      <c r="C48" s="25" t="n"/>
+      <c r="D48" s="25" t="n"/>
+      <c r="E48" s="25" t="n"/>
+      <c r="F48" s="25" t="n"/>
+      <c r="G48" s="25" t="n"/>
+      <c r="H48" s="25" t="n"/>
+      <c r="I48" s="25" t="n"/>
+      <c r="J48" s="25" t="n"/>
+      <c r="K48" s="26" t="n"/>
+      <c r="L48" s="14">
+        <f>L7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="22" t="inlineStr">
+        <is>
+          <t>Less: Attorney Fees</t>
+        </is>
+      </c>
+      <c r="C49" s="25" t="n"/>
+      <c r="D49" s="25" t="n"/>
+      <c r="E49" s="25" t="n"/>
+      <c r="F49" s="25" t="n"/>
+      <c r="G49" s="25" t="n"/>
+      <c r="H49" s="25" t="n"/>
+      <c r="I49" s="25" t="n"/>
+      <c r="J49" s="25" t="n"/>
+      <c r="K49" s="26" t="n"/>
+      <c r="L49" s="14">
+        <f>-L11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="B50" s="22" t="inlineStr">
+        <is>
+          <t>Less: Advanced Case Expenses</t>
+        </is>
+      </c>
+      <c r="C50" s="25" t="n"/>
+      <c r="D50" s="25" t="n"/>
+      <c r="E50" s="25" t="n"/>
+      <c r="F50" s="25" t="n"/>
+      <c r="G50" s="25" t="n"/>
+      <c r="H50" s="25" t="n"/>
+      <c r="I50" s="25" t="n"/>
+      <c r="J50" s="25" t="n"/>
+      <c r="K50" s="26" t="n"/>
+      <c r="L50" s="14">
+        <f>-L20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="B51" s="22" t="inlineStr">
+        <is>
+          <t>Less: Total Liens (Reduced)</t>
+        </is>
+      </c>
+      <c r="C51" s="25" t="n"/>
+      <c r="D51" s="25" t="n"/>
+      <c r="E51" s="25" t="n"/>
+      <c r="F51" s="25" t="n"/>
+      <c r="G51" s="25" t="n"/>
+      <c r="H51" s="25" t="n"/>
+      <c r="I51" s="25" t="n"/>
+      <c r="J51" s="25" t="n"/>
+      <c r="K51" s="26" t="n"/>
+      <c r="L51" s="14">
+        <f>-L44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="B52" s="28" t="inlineStr">
+        <is>
+          <t>NET CLIENT DISBURSEMENT</t>
+        </is>
+      </c>
+      <c r="C52" s="25" t="n"/>
+      <c r="D52" s="25" t="n"/>
+      <c r="E52" s="25" t="n"/>
+      <c r="F52" s="25" t="n"/>
+      <c r="G52" s="25" t="n"/>
+      <c r="H52" s="25" t="n"/>
+      <c r="I52" s="25" t="n"/>
+      <c r="J52" s="25" t="n"/>
+      <c r="K52" s="26" t="n"/>
+      <c r="L52" s="17">
+        <f>SUM(L48:L51)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="27">
+    <mergeCell ref="C16:K16"/>
+    <mergeCell ref="B49:K49"/>
+    <mergeCell ref="C10:K10"/>
+    <mergeCell ref="B46:L46"/>
+    <mergeCell ref="B51:K51"/>
+    <mergeCell ref="B20:K20"/>
+    <mergeCell ref="C12:K12"/>
+    <mergeCell ref="C11:K11"/>
+    <mergeCell ref="B50:K50"/>
+    <mergeCell ref="C17:K17"/>
+    <mergeCell ref="B47:K47"/>
+    <mergeCell ref="B23:L23"/>
+    <mergeCell ref="C7:K7"/>
+    <mergeCell ref="C19:K19"/>
+    <mergeCell ref="B52:K52"/>
+    <mergeCell ref="C13:K13"/>
+    <mergeCell ref="B21:K21"/>
+    <mergeCell ref="C18:K18"/>
+    <mergeCell ref="B41:G41"/>
+    <mergeCell ref="B48:K48"/>
+    <mergeCell ref="B9:L9"/>
+    <mergeCell ref="C6:K6"/>
+    <mergeCell ref="C15:K15"/>
+    <mergeCell ref="B44:H44"/>
+    <mergeCell ref="C14:K14"/>
+    <mergeCell ref="B5:L5"/>
+    <mergeCell ref="B2:L3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AG52"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
+  <cols>
+    <col width="3.14" customWidth="1" style="23" min="1" max="1"/>
+    <col width="30.86" customWidth="1" style="23" min="2" max="2"/>
+    <col width="31.14" customWidth="1" style="23" min="3" max="8"/>
+    <col width="21.57" customWidth="1" style="23" min="9" max="11"/>
+    <col width="44.43" customWidth="1" style="23" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve"> PRACTICE — John Doe v. Apex (Aggressive Casualty offer $45,000 per Email 2). Fill the yellow cells; verify every figure against the source documents.</t>
         </is>
       </c>

</xml_diff>